<commit_message>
Snapshot Taranis-People-Data-Collection.xlsx (25 May, post-Drive-edit)
</commit_message>
<xml_diff>
--- a/Taranis-People-Data-Collection.xlsx
+++ b/Taranis-People-Data-Collection.xlsx
@@ -1,31 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mark\Claude Cowork\Taranis Capital Website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F6592E9-A66B-4F45-A619-098F24152DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C187EC5-08D0-428A-9135-9CD47602A1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="People Directory" sheetId="1" r:id="rId1"/>
     <sheet name="Profile Images" sheetId="2" r:id="rId2"/>
-    <sheet name="Missing LinkedIn" sheetId="3" r:id="rId3"/>
+    <sheet name="Removed People" sheetId="5" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'People Directory'!$A$1:$Z$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'People Directory'!$A$1:$Z$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Removed People'!$A$1:$Z$5</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1184" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="437">
   <si>
     <t>Slug</t>
   </si>
@@ -719,10 +720,13 @@
     <t>mohammed-aljumah</t>
   </si>
   <si>
-    <t>Professor Mohammed Al Jumah</t>
+    <t>Prof. Mohamed Al Jumah</t>
   </si>
   <si>
     <t>Senior Advisor</t>
+  </si>
+  <si>
+    <t>mohammed-aljumah@taraniscapital.com</t>
   </si>
   <si>
     <t>/images/team/Mohammed-AlJumah-Headshot-600-650-277x300.png</t>
@@ -798,6 +802,9 @@
 His combination of corporate leadership, entrepreneurial experience, and cybersecurity expertise provides Taranis Capital with critical perspective on technology risk, digital transformation, and enterprise-grade security.</t>
   </si>
   <si>
+    <t>taraniscapital.com/team/osama-al-thanon</t>
+  </si>
+  <si>
     <t>Over 40 years in executive leadership and cybersecurity. Former ABB C-level executive with deep expertise in digital transformation, white-hat security, and AI ventures. Saudi Council of Engineers member.</t>
   </si>
   <si>
@@ -810,7 +817,7 @@
     <t>osama-al-zamil</t>
   </si>
   <si>
-    <t>HE Eng. Osama Al-Zamil</t>
+    <t>H.E. Eng. Osama Al-Zamil</t>
   </si>
   <si>
     <t>Board Advisor</t>
@@ -829,9 +836,6 @@
     <t>taraniscapital.com/board/osama-al-zamil</t>
   </si>
   <si>
-    <t>Chairman of Advisory Board</t>
-  </si>
-  <si>
     <t>Former Vice Minister of Industry and Mineral Resources, Saudi Arabia (2019-2023). Designed Saudi Arabia's National Industrial Strategy as part of Vision 2030. 20+ years of private sector executive experience.</t>
   </si>
   <si>
@@ -847,7 +851,7 @@
     <t>osama-bukhari</t>
   </si>
   <si>
-    <t>Osama Ben Saleh Bukhari</t>
+    <t>Osama BenSaleh Bukhari</t>
   </si>
   <si>
     <t>Chief Technical Officer</t>
@@ -1209,7 +1213,7 @@
     <t>abdullah-alawad</t>
   </si>
   <si>
-    <t>Dr Abdullah Alawad</t>
+    <t>Prof. Abdullah Alawad</t>
   </si>
   <si>
     <t>abdullah@taraniscapital.com</t>
@@ -1226,6 +1230,9 @@
     <t>taraniscapital.com/board/abdullah-alawad</t>
   </si>
   <si>
+    <t>More than 20 years of experience in biotech and biomedical R&amp;D, innovation and ecosystem development. Held senior executive leadership roles and led national initiatives, advanced technologies and industrial transformation efforts. Advisor and board member with a strong track record of scaling science-based ventures, forging strategic partnerships and delivering high-impact growth.</t>
+  </si>
+  <si>
     <t>qaisar-hamed-metawea</t>
   </si>
   <si>
@@ -1369,38 +1376,26 @@
     <t>Junaid-Kashir-600x650-277x300.jpg</t>
   </si>
   <si>
+    <t>Dr Abdullah Alawad</t>
+  </si>
+  <si>
     <t>Abdullah-Alawad-600x650-277x300.jpg</t>
   </si>
   <si>
     <t>Qaisar-Hamed-Metawea-600x650-277x300.jpg</t>
   </si>
   <si>
-    <t>Role</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>OK</t>
-  </si>
-  <si>
-    <t>Prof. Abdullah Alawad</t>
-  </si>
-  <si>
-    <t>More than 20 years of experience in biotech and biomedical R&amp;D, innovation and ecosystem development. Held senior executive leadership roles and led national initiatives, advanced technologies and industrial transformation efforts. Advisor and board member with a strong track record of scaling science-based ventures, forging strategic partnerships and delivering high-impact growth.</t>
-  </si>
-  <si>
-    <t>Chief Cybersecurity Officer</t>
-  </si>
-  <si>
-    <t>taraniscapital.com/team/osama-al-thanon</t>
+    <t>https://www.linkedin.com/in/osama-skywalker/</t>
+  </si>
+  <si>
+    <t>Chief Strategy Officer</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1417,6 +1412,14 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1466,8 +1469,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1490,14 +1494,15 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1798,86 +1803,114 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z37"/>
+  <dimension ref="A1:Z33"/>
   <sheetFormatPr defaultColWidth="18" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="135.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="77.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="43.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="26.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="228.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="42.21875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="248" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="27.21875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="40.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="235.109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="42.88671875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="255.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L1" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="M1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="Q1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="R1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="S1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="U1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="V1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="W1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="9" t="s">
+      <c r="X1" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="9" t="s">
+      <c r="Y1" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="9" t="s">
+      <c r="Z1" s="8" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2159,10 +2192,10 @@
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>28</v>
@@ -2171,13 +2204,13 @@
         <v>29</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>75</v>
+        <v>86</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>33</v>
@@ -2186,10 +2219,10 @@
         <v>34</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>33</v>
@@ -2198,51 +2231,39 @@
         <v>29</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P6" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>80</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="1"/>
       <c r="R6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S6" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>81</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="S6" s="4"/>
+      <c r="T6" s="1"/>
       <c r="U6" s="3" t="s">
         <v>33</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="X6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y6" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z6" s="1" t="s">
-        <v>83</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="Y6" s="4"/>
+      <c r="Z6" s="1"/>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>28</v>
@@ -2251,13 +2272,13 @@
         <v>29</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>87</v>
+        <v>95</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>33</v>
@@ -2266,38 +2287,38 @@
         <v>34</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>91</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="M7" s="4"/>
+      <c r="N7" s="1"/>
       <c r="O7" s="3" t="s">
         <v>37</v>
       </c>
       <c r="P7" s="4"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="S7" s="4"/>
-      <c r="T7" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="S7" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="T7" s="1" t="s">
+        <v>100</v>
+      </c>
       <c r="U7" s="3" t="s">
         <v>33</v>
       </c>
       <c r="V7" s="4" t="s">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="X7" s="3" t="s">
         <v>37</v>
@@ -2307,10 +2328,10 @@
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>28</v>
@@ -2319,13 +2340,13 @@
         <v>29</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>33</v>
@@ -2334,38 +2355,38 @@
         <v>34</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M8" s="4"/>
-      <c r="N8" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>110</v>
+      </c>
       <c r="O8" s="3" t="s">
         <v>37</v>
       </c>
       <c r="P8" s="4"/>
       <c r="Q8" s="1"/>
       <c r="R8" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S8" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>100</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="S8" s="4"/>
+      <c r="T8" s="1"/>
       <c r="U8" s="3" t="s">
         <v>33</v>
       </c>
       <c r="V8" s="4" t="s">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="X8" s="3" t="s">
         <v>37</v>
@@ -2375,25 +2396,25 @@
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>29</v>
+        <v>114</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>33</v>
@@ -2402,66 +2423,70 @@
         <v>34</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M9" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>110</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="M9" s="4"/>
+      <c r="N9" s="1"/>
       <c r="O9" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="P9" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>121</v>
+      </c>
       <c r="R9" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="S9" s="4"/>
-      <c r="T9" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="S9" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="T9" s="1" t="s">
+        <v>123</v>
+      </c>
       <c r="U9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V9" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="W9" s="1" t="s">
-        <v>111</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="V9" s="4"/>
+      <c r="W9" s="1"/>
       <c r="X9" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Y9" s="4"/>
-      <c r="Z9" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="Y9" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="Z9" s="1" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>114</v>
+        <v>29</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>116</v>
+        <v>127</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>33</v>
@@ -2470,10 +2495,10 @@
         <v>34</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>37</v>
@@ -2481,22 +2506,18 @@
       <c r="M10" s="4"/>
       <c r="N10" s="1"/>
       <c r="O10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P10" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="Q10" s="1" t="s">
-        <v>121</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="1"/>
       <c r="R10" s="3" t="s">
         <v>33</v>
       </c>
       <c r="S10" s="4" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="U10" s="3" t="s">
         <v>37</v>
@@ -2504,21 +2525,17 @@
       <c r="V10" s="4"/>
       <c r="W10" s="1"/>
       <c r="X10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y10" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="Z10" s="1" t="s">
-        <v>124</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="Y10" s="4"/>
+      <c r="Z10" s="1"/>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>28</v>
@@ -2527,13 +2544,13 @@
         <v>29</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>87</v>
+        <v>135</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>136</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>33</v>
@@ -2542,35 +2559,39 @@
         <v>34</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M11" s="4"/>
-      <c r="N11" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>140</v>
+      </c>
       <c r="O11" s="3" t="s">
         <v>37</v>
       </c>
       <c r="P11" s="4"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S11" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="T11" s="1" t="s">
-        <v>132</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="S11" s="4"/>
+      <c r="T11" s="1"/>
       <c r="U11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V11" s="4"/>
-      <c r="W11" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="V11" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="W11" s="1" t="s">
+        <v>141</v>
+      </c>
       <c r="X11" s="3" t="s">
         <v>37</v>
       </c>
@@ -2579,10 +2600,10 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>28</v>
@@ -2591,13 +2612,13 @@
         <v>29</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>33</v>
@@ -2606,10 +2627,10 @@
         <v>34</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>33</v>
@@ -2618,13 +2639,17 @@
         <v>29</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P12" s="4"/>
-      <c r="Q12" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="P12" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>151</v>
+      </c>
       <c r="R12" s="3" t="s">
         <v>37</v>
       </c>
@@ -2637,7 +2662,7 @@
         <v>29</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="X12" s="3" t="s">
         <v>37</v>
@@ -2647,10 +2672,10 @@
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>28</v>
@@ -2659,13 +2684,13 @@
         <v>29</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>33</v>
@@ -2674,43 +2699,35 @@
         <v>34</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="N13" s="1" t="s">
-        <v>149</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="M13" s="4"/>
+      <c r="N13" s="1"/>
       <c r="O13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P13" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="Q13" s="1" t="s">
-        <v>151</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="1"/>
       <c r="R13" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="S13" s="4"/>
-      <c r="T13" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="S13" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="T13" s="1" t="s">
+        <v>161</v>
+      </c>
       <c r="U13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="W13" s="1" t="s">
-        <v>152</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="V13" s="4"/>
+      <c r="W13" s="1"/>
       <c r="X13" s="3" t="s">
         <v>37</v>
       </c>
@@ -2719,25 +2736,25 @@
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>29</v>
+        <v>164</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>33</v>
@@ -2746,62 +2763,78 @@
         <v>34</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M14" s="4"/>
-      <c r="N14" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="M14" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>170</v>
+      </c>
       <c r="O14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P14" s="4"/>
-      <c r="Q14" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="Q14" s="1" t="s">
+        <v>171</v>
+      </c>
       <c r="R14" s="3" t="s">
         <v>33</v>
       </c>
       <c r="S14" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="T14" s="1" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="U14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V14" s="4"/>
-      <c r="W14" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="V14" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="W14" s="1" t="s">
+        <v>173</v>
+      </c>
       <c r="X14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Y14" s="4"/>
-      <c r="Z14" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="Y14" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="Z14" s="1" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>164</v>
+        <v>29</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>33</v>
@@ -2810,63 +2843,55 @@
         <v>34</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M15" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="N15" s="1" t="s">
-        <v>170</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="M15" s="4"/>
+      <c r="N15" s="1"/>
       <c r="O15" s="3" t="s">
         <v>33</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="R15" s="3" t="s">
         <v>33</v>
       </c>
       <c r="S15" s="4" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="T15" s="1" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="U15" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V15" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="W15" s="1" t="s">
-        <v>173</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="V15" s="4"/>
+      <c r="W15" s="1"/>
       <c r="X15" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Y15" s="4" t="s">
-        <v>164</v>
+        <v>184</v>
       </c>
       <c r="Z15" s="1" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>28</v>
@@ -2875,13 +2900,13 @@
         <v>29</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>33</v>
@@ -2890,70 +2915,78 @@
         <v>34</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M16" s="4"/>
-      <c r="N16" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="M16" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>193</v>
+      </c>
       <c r="O16" s="3" t="s">
         <v>33</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="R16" s="3" t="s">
         <v>33</v>
       </c>
       <c r="S16" s="4" t="s">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="T16" s="1" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="U16" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V16" s="4"/>
-      <c r="W16" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="V16" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="W16" s="1" t="s">
+        <v>196</v>
+      </c>
       <c r="X16" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Y16" s="4" t="s">
-        <v>184</v>
+        <v>50</v>
       </c>
       <c r="Z16" s="1" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>29</v>
+        <v>200</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>33</v>
@@ -2962,78 +2995,66 @@
         <v>34</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M17" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="N17" s="1" t="s">
-        <v>193</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="M17" s="4"/>
+      <c r="N17" s="1"/>
       <c r="O17" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P17" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q17" s="1" t="s">
-        <v>194</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="P17" s="4"/>
+      <c r="Q17" s="1"/>
       <c r="R17" s="3" t="s">
         <v>33</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="T17" s="1" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="U17" s="3" t="s">
         <v>33</v>
       </c>
       <c r="V17" s="4" t="s">
-        <v>29</v>
+        <v>207</v>
       </c>
       <c r="W17" s="1" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="X17" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y17" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z17" s="1" t="s">
-        <v>197</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="Y17" s="4"/>
+      <c r="Z17" s="1"/>
     </row>
     <row r="18" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>33</v>
@@ -3042,66 +3063,78 @@
         <v>34</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M18" s="4"/>
-      <c r="N18" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="M18" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>218</v>
+      </c>
       <c r="O18" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P18" s="4"/>
-      <c r="Q18" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="P18" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="Q18" s="1" t="s">
+        <v>219</v>
+      </c>
       <c r="R18" s="3" t="s">
         <v>33</v>
       </c>
       <c r="S18" s="4" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="T18" s="1" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="U18" s="3" t="s">
         <v>33</v>
       </c>
       <c r="V18" s="4" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="W18" s="1" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="X18" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Y18" s="4"/>
-      <c r="Z18" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="Y18" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="Z18" s="1" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="19" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>213</v>
+        <v>226</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>33</v>
@@ -3110,76 +3143,62 @@
         <v>34</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M19" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="N19" s="1" t="s">
-        <v>218</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="M19" s="4"/>
+      <c r="N19" s="1"/>
       <c r="O19" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P19" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="Q19" s="1" t="s">
-        <v>219</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="P19" s="4"/>
+      <c r="Q19" s="1"/>
       <c r="R19" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S19" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="T19" s="1" t="s">
-        <v>220</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="S19" s="4"/>
+      <c r="T19" s="1"/>
       <c r="U19" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V19" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="W19" s="1" t="s">
-        <v>221</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="V19" s="4"/>
+      <c r="W19" s="1"/>
       <c r="X19" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Y19" s="4" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="Z19" s="1" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
     </row>
     <row r="20" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="5" t="s">
-        <v>87</v>
+        <v>234</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>236</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>33</v>
@@ -3188,62 +3207,78 @@
         <v>34</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M20" s="4"/>
-      <c r="N20" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="N20" s="1" t="s">
+        <v>240</v>
+      </c>
       <c r="O20" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P20" s="4"/>
-      <c r="Q20" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="P20" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q20" s="1" t="s">
+        <v>241</v>
+      </c>
       <c r="R20" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="S20" s="4"/>
-      <c r="T20" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="S20" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="T20" s="1" t="s">
+        <v>242</v>
+      </c>
       <c r="U20" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V20" s="4"/>
-      <c r="W20" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="V20" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="W20" s="1" t="s">
+        <v>240</v>
+      </c>
       <c r="X20" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Y20" s="4" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="Z20" s="1" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
     </row>
     <row r="21" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>231</v>
+        <v>245</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>233</v>
+        <v>436</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>235</v>
+        <v>247</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>435</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>33</v>
@@ -3252,78 +3287,74 @@
         <v>34</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="L21" s="3" t="s">
         <v>33</v>
       </c>
       <c r="M21" s="4" t="s">
-        <v>233</v>
+        <v>256</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P21" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="Q21" s="1" t="s">
-        <v>240</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="P21" s="4"/>
+      <c r="Q21" s="1"/>
       <c r="R21" s="3" t="s">
         <v>33</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>233</v>
+        <v>131</v>
       </c>
       <c r="T21" s="1" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="U21" s="3" t="s">
         <v>33</v>
       </c>
       <c r="V21" s="4" t="s">
-        <v>233</v>
+        <v>29</v>
       </c>
       <c r="W21" s="1" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="X21" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Y21" s="4" t="s">
-        <v>242</v>
+        <v>50</v>
       </c>
       <c r="Z21" s="1" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>437</v>
+        <v>256</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>246</v>
+        <v>257</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>247</v>
+        <v>258</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>33</v>
@@ -3332,42 +3363,42 @@
         <v>34</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>248</v>
+        <v>259</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>438</v>
+        <v>260</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M22" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="N22" s="1" t="s">
-        <v>249</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="M22" s="4"/>
+      <c r="N22" s="1"/>
       <c r="O22" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P22" s="4"/>
-      <c r="Q22" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="P22" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q22" s="1" t="s">
+        <v>261</v>
+      </c>
       <c r="R22" s="3" t="s">
         <v>33</v>
       </c>
       <c r="S22" s="4" t="s">
-        <v>131</v>
+        <v>50</v>
       </c>
       <c r="T22" s="1" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
       <c r="U22" s="3" t="s">
         <v>33</v>
       </c>
       <c r="V22" s="4" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="W22" s="1" t="s">
-        <v>250</v>
+        <v>263</v>
       </c>
       <c r="X22" s="3" t="s">
         <v>33</v>
@@ -3376,30 +3407,30 @@
         <v>50</v>
       </c>
       <c r="Z22" s="1" t="s">
-        <v>251</v>
+        <v>264</v>
       </c>
     </row>
     <row r="23" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>87</v>
+        <v>268</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>269</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>33</v>
@@ -3408,74 +3439,78 @@
         <v>34</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>257</v>
+        <v>271</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M23" s="4"/>
-      <c r="N23" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="M23" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>273</v>
+      </c>
       <c r="O23" s="3" t="s">
         <v>33</v>
       </c>
       <c r="P23" s="4" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="Q23" s="1" t="s">
-        <v>260</v>
+        <v>274</v>
       </c>
       <c r="R23" s="3" t="s">
         <v>33</v>
       </c>
       <c r="S23" s="4" t="s">
-        <v>259</v>
+        <v>275</v>
       </c>
       <c r="T23" s="1" t="s">
-        <v>261</v>
+        <v>276</v>
       </c>
       <c r="U23" s="3" t="s">
         <v>33</v>
       </c>
       <c r="V23" s="4" t="s">
-        <v>29</v>
+        <v>267</v>
       </c>
       <c r="W23" s="1" t="s">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="X23" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Y23" s="4" t="s">
-        <v>50</v>
+        <v>278</v>
       </c>
       <c r="Z23" s="1" t="s">
-        <v>263</v>
+        <v>279</v>
       </c>
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>265</v>
+        <v>281</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>266</v>
+        <v>29</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>267</v>
+        <v>282</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>268</v>
+        <v>283</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>269</v>
+        <v>284</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>33</v>
@@ -3484,63 +3519,51 @@
         <v>34</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>270</v>
+        <v>285</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>271</v>
+        <v>286</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M24" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="N24" s="1" t="s">
-        <v>272</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="M24" s="4"/>
+      <c r="N24" s="1"/>
       <c r="O24" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P24" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="Q24" s="1" t="s">
-        <v>273</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="1"/>
       <c r="R24" s="3" t="s">
         <v>33</v>
       </c>
       <c r="S24" s="4" t="s">
-        <v>274</v>
+        <v>50</v>
       </c>
       <c r="T24" s="1" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="U24" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V24" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="W24" s="1" t="s">
-        <v>276</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="V24" s="4"/>
+      <c r="W24" s="1"/>
       <c r="X24" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Y24" s="4" t="s">
-        <v>277</v>
+        <v>50</v>
       </c>
       <c r="Z24" s="1" t="s">
-        <v>278</v>
+        <v>288</v>
       </c>
     </row>
     <row r="25" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>279</v>
+        <v>289</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>280</v>
+        <v>290</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>28</v>
@@ -3549,13 +3572,13 @@
         <v>29</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>281</v>
+        <v>291</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="H25" s="2" t="s">
         <v>33</v>
@@ -3564,66 +3587,66 @@
         <v>34</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>285</v>
+        <v>295</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M25" s="4"/>
-      <c r="N25" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="M25" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>297</v>
+      </c>
       <c r="O25" s="3" t="s">
         <v>37</v>
       </c>
       <c r="P25" s="4"/>
       <c r="Q25" s="1"/>
       <c r="R25" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S25" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="T25" s="1" t="s">
-        <v>286</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="S25" s="4"/>
+      <c r="T25" s="1"/>
       <c r="U25" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V25" s="4"/>
-      <c r="W25" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="V25" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="W25" s="1" t="s">
+        <v>298</v>
+      </c>
       <c r="X25" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y25" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z25" s="1" t="s">
-        <v>287</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="Y25" s="4"/>
+      <c r="Z25" s="1"/>
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>288</v>
+        <v>299</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>289</v>
+        <v>300</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>29</v>
+        <v>301</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>33</v>
@@ -3632,20 +3655,16 @@
         <v>34</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M26" s="4" t="s">
-        <v>295</v>
-      </c>
-      <c r="N26" s="1" t="s">
-        <v>296</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="M26" s="4"/>
+      <c r="N26" s="1"/>
       <c r="O26" s="3" t="s">
         <v>37</v>
       </c>
@@ -3660,10 +3679,10 @@
         <v>33</v>
       </c>
       <c r="V26" s="4" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="W26" s="1" t="s">
-        <v>297</v>
+        <v>307</v>
       </c>
       <c r="X26" s="3" t="s">
         <v>37</v>
@@ -3673,25 +3692,25 @@
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>299</v>
+        <v>309</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>300</v>
+        <v>29</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="H27" s="2" t="s">
         <v>33</v>
@@ -3700,10 +3719,10 @@
         <v>34</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>304</v>
+        <v>313</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>305</v>
+        <v>314</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>37</v>
@@ -3724,38 +3743,42 @@
         <v>33</v>
       </c>
       <c r="V27" s="4" t="s">
-        <v>300</v>
+        <v>315</v>
       </c>
       <c r="W27" s="1" t="s">
-        <v>306</v>
+        <v>316</v>
       </c>
       <c r="X27" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Y27" s="4"/>
-      <c r="Z27" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="Y27" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="Z27" s="1" t="s">
+        <v>318</v>
+      </c>
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>307</v>
+        <v>338</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>308</v>
+        <v>339</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>29</v>
+        <v>340</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>309</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>310</v>
+        <v>341</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>311</v>
+        <v>342</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>33</v>
@@ -3764,10 +3787,10 @@
         <v>34</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>312</v>
+        <v>343</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>313</v>
+        <v>344</v>
       </c>
       <c r="L28" s="3" t="s">
         <v>37</v>
@@ -3785,45 +3808,41 @@
       <c r="S28" s="4"/>
       <c r="T28" s="1"/>
       <c r="U28" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V28" s="4" t="s">
-        <v>314</v>
-      </c>
-      <c r="W28" s="1" t="s">
-        <v>315</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="V28" s="4"/>
+      <c r="W28" s="1"/>
       <c r="X28" s="3" t="s">
         <v>33</v>
       </c>
       <c r="Y28" s="4" t="s">
-        <v>316</v>
+        <v>340</v>
       </c>
       <c r="Z28" s="1" t="s">
-        <v>317</v>
+        <v>345</v>
       </c>
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>318</v>
+        <v>346</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>319</v>
+        <v>347</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>101</v>
+        <v>28</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>320</v>
+        <v>340</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>321</v>
+        <v>348</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>322</v>
+        <v>349</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>323</v>
+        <v>350</v>
       </c>
       <c r="H29" s="2" t="s">
         <v>33</v>
@@ -3832,10 +3851,10 @@
         <v>34</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>324</v>
+        <v>351</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>325</v>
+        <v>352</v>
       </c>
       <c r="L29" s="3" t="s">
         <v>37</v>
@@ -3848,14 +3867,10 @@
       <c r="P29" s="4"/>
       <c r="Q29" s="1"/>
       <c r="R29" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S29" s="4" t="s">
-        <v>320</v>
-      </c>
-      <c r="T29" s="1" t="s">
-        <v>326</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="S29" s="4"/>
+      <c r="T29" s="1"/>
       <c r="U29" s="3" t="s">
         <v>37</v>
       </c>
@@ -3865,33 +3880,33 @@
         <v>33</v>
       </c>
       <c r="Y29" s="4" t="s">
-        <v>320</v>
+        <v>340</v>
       </c>
       <c r="Z29" s="1" t="s">
-        <v>327</v>
+        <v>353</v>
       </c>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>328</v>
+        <v>354</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>329</v>
+        <v>355</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>101</v>
+        <v>28</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>330</v>
+        <v>356</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>331</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>87</v>
+        <v>357</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>358</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>332</v>
+        <v>359</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>33</v>
@@ -3900,10 +3915,10 @@
         <v>34</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>333</v>
+        <v>360</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>334</v>
+        <v>361</v>
       </c>
       <c r="L30" s="3" t="s">
         <v>37</v>
@@ -3916,14 +3931,10 @@
       <c r="P30" s="4"/>
       <c r="Q30" s="1"/>
       <c r="R30" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S30" s="4" t="s">
-        <v>330</v>
-      </c>
-      <c r="T30" s="1" t="s">
-        <v>335</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="S30" s="4"/>
+      <c r="T30" s="1"/>
       <c r="U30" s="3" t="s">
         <v>37</v>
       </c>
@@ -3933,33 +3944,33 @@
         <v>33</v>
       </c>
       <c r="Y30" s="4" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="Z30" s="1" t="s">
-        <v>336</v>
+        <v>362</v>
       </c>
     </row>
     <row r="31" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>337</v>
+        <v>363</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>338</v>
+        <v>364</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>340</v>
+        <v>366</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>33</v>
@@ -3968,10 +3979,10 @@
         <v>34</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>343</v>
+        <v>369</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>37</v>
@@ -3997,33 +4008,33 @@
         <v>33</v>
       </c>
       <c r="Y31" s="4" t="s">
-        <v>339</v>
+        <v>38</v>
       </c>
       <c r="Z31" s="1" t="s">
-        <v>344</v>
+        <v>370</v>
       </c>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>345</v>
+        <v>371</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>346</v>
+        <v>372</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>347</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>348</v>
+        <v>373</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>349</v>
+        <v>374</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>33</v>
@@ -4032,10 +4043,10 @@
         <v>34</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>350</v>
+        <v>375</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>351</v>
+        <v>376</v>
       </c>
       <c r="L32" s="3" t="s">
         <v>37</v>
@@ -4061,33 +4072,33 @@
         <v>33</v>
       </c>
       <c r="Y32" s="4" t="s">
-        <v>339</v>
+        <v>38</v>
       </c>
       <c r="Z32" s="1" t="s">
-        <v>352</v>
+        <v>377</v>
       </c>
     </row>
     <row r="33" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>353</v>
+        <v>378</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>354</v>
+        <v>379</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>356</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>357</v>
+        <v>380</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>358</v>
+        <v>381</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>33</v>
@@ -4096,10 +4107,10 @@
         <v>34</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>359</v>
+        <v>382</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>360</v>
+        <v>383</v>
       </c>
       <c r="L33" s="3" t="s">
         <v>37</v>
@@ -4125,274 +4136,17 @@
         <v>33</v>
       </c>
       <c r="Y33" s="4" t="s">
-        <v>339</v>
+        <v>38</v>
       </c>
       <c r="Z33" s="1" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
-        <v>362</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>363</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>364</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>366</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="K34" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="L34" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M34" s="4"/>
-      <c r="N34" s="1"/>
-      <c r="O34" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P34" s="4"/>
-      <c r="Q34" s="1"/>
-      <c r="R34" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="S34" s="4"/>
-      <c r="T34" s="1"/>
-      <c r="U34" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V34" s="4"/>
-      <c r="W34" s="1"/>
-      <c r="X34" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y34" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z34" s="1" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>371</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>364</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>373</v>
-      </c>
-      <c r="H35" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>374</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>375</v>
-      </c>
-      <c r="L35" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M35" s="4"/>
-      <c r="N35" s="1"/>
-      <c r="O35" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P35" s="4"/>
-      <c r="Q35" s="1"/>
-      <c r="R35" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="S35" s="4"/>
-      <c r="T35" s="1"/>
-      <c r="U35" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V35" s="4"/>
-      <c r="W35" s="1"/>
-      <c r="X35" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y35" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z35" s="1" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
-        <v>377</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>364</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>379</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>380</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I36" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J36" s="1" t="s">
-        <v>381</v>
-      </c>
-      <c r="K36" s="1" t="s">
-        <v>382</v>
-      </c>
-      <c r="L36" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M36" s="4"/>
-      <c r="N36" s="1"/>
-      <c r="O36" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P36" s="4"/>
-      <c r="Q36" s="1"/>
-      <c r="R36" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="S36" s="4"/>
-      <c r="T36" s="1"/>
-      <c r="U36" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V36" s="4"/>
-      <c r="W36" s="1"/>
-      <c r="X36" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y36" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z36" s="1" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
-        <v>383</v>
-      </c>
-      <c r="B37" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>385</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>386</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>387</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I37" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>388</v>
-      </c>
-      <c r="K37" s="1" t="s">
-        <v>389</v>
-      </c>
-      <c r="L37" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M37" s="4"/>
-      <c r="N37" s="1"/>
-      <c r="O37" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P37" s="4"/>
-      <c r="Q37" s="1"/>
-      <c r="R37" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S37" s="4" t="s">
-        <v>390</v>
-      </c>
-      <c r="T37" s="1" t="s">
-        <v>391</v>
-      </c>
-      <c r="U37" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V37" s="4"/>
-      <c r="W37" s="1"/>
-      <c r="X37" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y37" s="4" t="s">
-        <v>390</v>
-      </c>
-      <c r="Z37" s="1" t="s">
-        <v>392</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z37" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:Z33" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <hyperlinks>
+    <hyperlink ref="F21" r:id="rId1" xr:uid="{EA65C852-03F8-4014-BA8C-24F049A82987}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4417,13 +4171,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -4434,7 +4188,7 @@
         <v>27</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>32</v>
@@ -4451,7 +4205,7 @@
         <v>41</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>46</v>
@@ -4468,7 +4222,7 @@
         <v>54</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>57</v>
@@ -4485,7 +4239,7 @@
         <v>65</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>69</v>
@@ -4502,7 +4256,7 @@
         <v>73</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>76</v>
@@ -4519,7 +4273,7 @@
         <v>85</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>88</v>
@@ -4536,7 +4290,7 @@
         <v>94</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>97</v>
@@ -4553,7 +4307,7 @@
         <v>104</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>107</v>
@@ -4570,7 +4324,7 @@
         <v>113</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>117</v>
@@ -4587,7 +4341,7 @@
         <v>126</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>128</v>
@@ -4604,7 +4358,7 @@
         <v>134</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>137</v>
@@ -4621,7 +4375,7 @@
         <v>143</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>146</v>
@@ -4638,7 +4392,7 @@
         <v>154</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>157</v>
@@ -4655,7 +4409,7 @@
         <v>163</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>167</v>
@@ -4672,7 +4426,7 @@
         <v>176</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>179</v>
@@ -4689,7 +4443,7 @@
         <v>187</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>190</v>
@@ -4706,7 +4460,7 @@
         <v>199</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>203</v>
@@ -4723,7 +4477,7 @@
         <v>210</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>214</v>
@@ -4740,10 +4494,10 @@
         <v>224</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>33</v>
@@ -4751,16 +4505,16 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>33</v>
@@ -4768,16 +4522,16 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>33</v>
@@ -4785,16 +4539,16 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>33</v>
@@ -4802,16 +4556,16 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>33</v>
@@ -4819,16 +4573,16 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>33</v>
@@ -4836,16 +4590,16 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>33</v>
@@ -4853,16 +4607,16 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>33</v>
@@ -4870,16 +4624,16 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>33</v>
@@ -4887,16 +4641,16 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E29" s="7" t="s">
         <v>33</v>
@@ -4904,16 +4658,16 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>33</v>
@@ -4921,16 +4675,16 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E31" s="7" t="s">
         <v>33</v>
@@ -4938,16 +4692,16 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E32" s="7" t="s">
         <v>33</v>
@@ -4955,16 +4709,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E33" s="7" t="s">
         <v>33</v>
@@ -4972,16 +4726,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>33</v>
@@ -4989,16 +4743,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>33</v>
@@ -5006,16 +4760,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>378</v>
+        <v>432</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>33</v>
@@ -5023,16 +4777,16 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="E37" s="7" t="s">
         <v>33</v>
@@ -5044,759 +4798,404 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D0D2A81-9E76-4402-B61B-4BC80E0978A0}">
+  <dimension ref="A1:Z5"/>
+  <sheetFormatPr defaultColWidth="18" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="35" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="55" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="135.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="77.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="43.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="26.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="228.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="42.21875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="248" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="27.21875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="40.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="235.109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="42.88671875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="255.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
-        <v>432</v>
-      </c>
-      <c r="E1" s="6" t="s">
+      <c r="D1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="6" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="G1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="E2" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="4" t="s">
+      <c r="N2" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="V2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" s="4"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="U3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="V3" s="4"/>
+      <c r="W3" s="1"/>
+      <c r="X3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y3" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="G4" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4" s="4"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S4" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="V4" s="4"/>
+      <c r="W4" s="1"/>
+      <c r="X4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y4" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="Z4" s="1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
-        <v>279</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>282</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
-        <v>288</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>289</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>291</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
-        <v>298</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>299</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>300</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="F28" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
-        <v>318</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>319</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>320</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>322</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>329</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>330</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
-        <v>337</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>339</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F31" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
-        <v>345</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>346</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>339</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>348</v>
-      </c>
-      <c r="F32" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>354</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>355</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>357</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="4" t="s">
-        <v>362</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>363</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>364</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="4" t="s">
-        <v>370</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>371</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>364</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="4" t="s">
-        <v>377</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>378</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>364</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F36" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="4" t="s">
-        <v>383</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>384</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>385</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F37" s="8" t="s">
-        <v>87</v>
+      <c r="G5" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" s="4"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S5" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="U5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="V5" s="4"/>
+      <c r="W5" s="1"/>
+      <c r="X5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y5" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="Z5" s="1" t="s">
+        <v>394</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:Z5" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly sync 2026-06-09: Osama Al-Zamil bio title, two Legal Counsel fixes, Osama Al-Thanon email
</commit_message>
<xml_diff>
--- a/Taranis-People-Data-Collection.xlsx
+++ b/Taranis-People-Data-Collection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mark\Claude Cowork\Taranis Capital Website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C187EC5-08D0-428A-9135-9CD47602A1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7AEFF62-1B67-497A-B4C9-6606C5236166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="People Directory" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="435">
   <si>
     <t>Slug</t>
   </si>
@@ -384,9 +384,6 @@
     <t>Emad Zowawi</t>
   </si>
   <si>
-    <t>KSA Legal Consul to the CEO</t>
-  </si>
-  <si>
     <t>emad@taraniscapital.com</t>
   </si>
   <si>
@@ -681,9 +678,6 @@
     <t>Mohamed Essam</t>
   </si>
   <si>
-    <t>Legal Consul</t>
-  </si>
-  <si>
     <t>mohamed@taraniscapital.com</t>
   </si>
   <si>
@@ -829,10 +823,6 @@
     <t>/images/team/His-Excellency-Eng.-Osama-Abdulaziz-Al-Zamil-Joins-600x650-1-277x300.png</t>
   </si>
   <si>
-    <t>Osama Al-Zamil is Chairman of the Advisory Board at Taranis Capital. He is a distinguished Saudi industrial leader with a remarkable career spanning multiple decades in business, government, and strategic advisory roles.
-His extensive experience includes senior government positions, including former Vice Minister of Industry, as well as leadership roles in major Saudi industrial and commercial enterprises. He brings unparalleled expertise in MENA markets, industrial development, international trade, and strategic capital deployment.</t>
-  </si>
-  <si>
     <t>taraniscapital.com/board/osama-al-zamil</t>
   </si>
   <si>
@@ -1389,6 +1379,10 @@
   </si>
   <si>
     <t>Chief Strategy Officer</t>
+  </si>
+  <si>
+    <t>Osama Al-Zamil is a Board Adviser at Taranis Capital. He is a distinguished Saudi industrial leader with a remarkable career spanning multiple decades in business, government, and strategic advisory roles.
+His extensive experience includes senior government positions, including former Vice Minister of Industry, as well as leadership roles in major Saudi industrial and commercial enterprises. He brings unparalleled expertise in MENA markets, industrial development, international trade, and strategic capital deployment.</t>
   </si>
 </sst>
 </file>
@@ -2405,16 +2399,16 @@
         <v>42</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>33</v>
@@ -2423,10 +2417,10 @@
         <v>34</v>
       </c>
       <c r="J9" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="K9" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>37</v>
@@ -2437,19 +2431,19 @@
         <v>33</v>
       </c>
       <c r="P9" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q9" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="Q9" s="1" t="s">
+      <c r="R9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S9" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="R9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S9" s="4" t="s">
+      <c r="T9" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>123</v>
       </c>
       <c r="U9" s="3" t="s">
         <v>37</v>
@@ -2460,18 +2454,18 @@
         <v>33</v>
       </c>
       <c r="Y9" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="Z9" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>126</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>28</v>
@@ -2480,13 +2474,13 @@
         <v>29</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>33</v>
@@ -2495,10 +2489,10 @@
         <v>34</v>
       </c>
       <c r="J10" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="K10" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>130</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>37</v>
@@ -2514,10 +2508,10 @@
         <v>33</v>
       </c>
       <c r="S10" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="T10" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="T10" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="U10" s="3" t="s">
         <v>37</v>
@@ -2532,10 +2526,10 @@
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>134</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>28</v>
@@ -2544,13 +2538,13 @@
         <v>29</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>137</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>33</v>
@@ -2559,10 +2553,10 @@
         <v>34</v>
       </c>
       <c r="J11" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="K11" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>139</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>33</v>
@@ -2571,7 +2565,7 @@
         <v>29</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O11" s="3" t="s">
         <v>37</v>
@@ -2590,7 +2584,7 @@
         <v>29</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="X11" s="3" t="s">
         <v>37</v>
@@ -2600,10 +2594,10 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>143</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>28</v>
@@ -2612,13 +2606,13 @@
         <v>29</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>33</v>
@@ -2627,10 +2621,10 @@
         <v>34</v>
       </c>
       <c r="J12" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="K12" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>148</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>33</v>
@@ -2639,16 +2633,16 @@
         <v>29</v>
       </c>
       <c r="N12" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P12" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="O12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P12" s="4" t="s">
+      <c r="Q12" s="1" t="s">
         <v>150</v>
-      </c>
-      <c r="Q12" s="1" t="s">
-        <v>151</v>
       </c>
       <c r="R12" s="3" t="s">
         <v>37</v>
@@ -2662,7 +2656,7 @@
         <v>29</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="X12" s="3" t="s">
         <v>37</v>
@@ -2672,10 +2666,10 @@
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>28</v>
@@ -2684,13 +2678,13 @@
         <v>29</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>156</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>157</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>33</v>
@@ -2699,10 +2693,10 @@
         <v>34</v>
       </c>
       <c r="J13" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="K13" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="L13" s="3" t="s">
         <v>37</v>
@@ -2718,10 +2712,10 @@
         <v>33</v>
       </c>
       <c r="S13" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="T13" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="T13" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="U13" s="3" t="s">
         <v>37</v>
@@ -2736,25 +2730,25 @@
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>163</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>167</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>33</v>
@@ -2763,63 +2757,63 @@
         <v>34</v>
       </c>
       <c r="J14" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="K14" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="L14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M14" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="N14" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="L14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M14" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="N14" s="1" t="s">
+      <c r="O14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q14" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="O14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P14" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="Q14" s="1" t="s">
+      <c r="R14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S14" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="T14" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="R14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S14" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="T14" s="1" t="s">
+      <c r="U14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="V14" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="W14" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="U14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V14" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="W14" s="1" t="s">
+      <c r="X14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y14" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="Z14" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="X14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y14" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="Z14" s="1" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>176</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>28</v>
@@ -2828,13 +2822,13 @@
         <v>29</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>179</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>33</v>
@@ -2843,10 +2837,10 @@
         <v>34</v>
       </c>
       <c r="J15" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="K15" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>181</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>37</v>
@@ -2857,19 +2851,19 @@
         <v>33</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="Q15" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="R15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S15" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="T15" s="1" t="s">
         <v>182</v>
-      </c>
-      <c r="R15" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S15" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="T15" s="1" t="s">
-        <v>183</v>
       </c>
       <c r="U15" s="3" t="s">
         <v>37</v>
@@ -2880,18 +2874,18 @@
         <v>33</v>
       </c>
       <c r="Y15" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="Z15" s="1" t="s">
         <v>184</v>
-      </c>
-      <c r="Z15" s="1" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>186</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>187</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>28</v>
@@ -2900,13 +2894,13 @@
         <v>29</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>33</v>
@@ -2915,10 +2909,10 @@
         <v>34</v>
       </c>
       <c r="J16" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="K16" s="1" t="s">
         <v>191</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>33</v>
@@ -2927,7 +2921,7 @@
         <v>29</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O16" s="3" t="s">
         <v>33</v>
@@ -2936,7 +2930,7 @@
         <v>50</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="R16" s="3" t="s">
         <v>33</v>
@@ -2945,7 +2939,7 @@
         <v>50</v>
       </c>
       <c r="T16" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="U16" s="3" t="s">
         <v>33</v>
@@ -2954,7 +2948,7 @@
         <v>29</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="X16" s="3" t="s">
         <v>33</v>
@@ -2963,30 +2957,30 @@
         <v>50</v>
       </c>
       <c r="Z16" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>198</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>199</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>33</v>
@@ -2995,10 +2989,10 @@
         <v>34</v>
       </c>
       <c r="J17" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="K17" s="1" t="s">
         <v>204</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>205</v>
       </c>
       <c r="L17" s="3" t="s">
         <v>37</v>
@@ -3014,19 +3008,19 @@
         <v>33</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="T17" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="U17" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="V17" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="U17" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V17" s="4" t="s">
+      <c r="W17" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="W17" s="1" t="s">
-        <v>208</v>
       </c>
       <c r="X17" s="3" t="s">
         <v>37</v>
@@ -3036,25 +3030,25 @@
     </row>
     <row r="18" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>210</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>214</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>33</v>
@@ -3063,78 +3057,78 @@
         <v>34</v>
       </c>
       <c r="J18" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M18" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="N18" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="L18" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M18" s="4" t="s">
+      <c r="O18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P18" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q18" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="N18" s="1" t="s">
+      <c r="R18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S18" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="T18" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="O18" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P18" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="Q18" s="1" t="s">
+      <c r="U18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="V18" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="W18" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="R18" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S18" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="T18" s="1" t="s">
+      <c r="X18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y18" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="Z18" s="1" t="s">
         <v>220</v>
-      </c>
-      <c r="U18" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V18" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="W18" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="X18" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y18" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="Z18" s="1" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="19" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>33</v>
@@ -3143,10 +3137,10 @@
         <v>34</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>37</v>
@@ -3172,33 +3166,33 @@
         <v>33</v>
       </c>
       <c r="Y19" s="4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="Z19" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="20" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>235</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>33</v>
@@ -3207,78 +3201,78 @@
         <v>34</v>
       </c>
       <c r="J20" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="N20" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="K20" s="1" t="s">
+      <c r="O20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P20" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="Q20" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="L20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M20" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="N20" s="1" t="s">
+      <c r="R20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S20" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="T20" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="O20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P20" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="Q20" s="1" t="s">
+      <c r="U20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="V20" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="W20" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="X20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y20" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="R20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S20" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="T20" s="1" t="s">
+      <c r="Z20" s="1" t="s">
         <v>242</v>
-      </c>
-      <c r="U20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V20" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="W20" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="X20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y20" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="Z20" s="1" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="21" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>33</v>
@@ -3287,19 +3281,19 @@
         <v>34</v>
       </c>
       <c r="J21" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M21" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="N21" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="L21" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M21" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="N21" s="1" t="s">
-        <v>251</v>
       </c>
       <c r="O21" s="3" t="s">
         <v>37</v>
@@ -3310,10 +3304,10 @@
         <v>33</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="T21" s="1" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="U21" s="3" t="s">
         <v>33</v>
@@ -3322,7 +3316,7 @@
         <v>29</v>
       </c>
       <c r="W21" s="1" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="X21" s="3" t="s">
         <v>33</v>
@@ -3331,30 +3325,30 @@
         <v>50</v>
       </c>
       <c r="Z21" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>33</v>
@@ -3363,10 +3357,10 @@
         <v>34</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>259</v>
+        <v>434</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="L22" s="3" t="s">
         <v>37</v>
@@ -3380,7 +3374,7 @@
         <v>50</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="R22" s="3" t="s">
         <v>33</v>
@@ -3389,7 +3383,7 @@
         <v>50</v>
       </c>
       <c r="T22" s="1" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="U22" s="3" t="s">
         <v>33</v>
@@ -3398,7 +3392,7 @@
         <v>50</v>
       </c>
       <c r="W22" s="1" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="X22" s="3" t="s">
         <v>33</v>
@@ -3407,30 +3401,30 @@
         <v>50</v>
       </c>
       <c r="Z22" s="1" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="23" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="G23" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>270</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>33</v>
@@ -3439,63 +3433,63 @@
         <v>34</v>
       </c>
       <c r="J23" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M23" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="O23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P23" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="Q23" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="K23" s="1" t="s">
+      <c r="R23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S23" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="L23" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M23" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="N23" s="1" t="s">
+      <c r="T23" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="O23" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P23" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="Q23" s="1" t="s">
+      <c r="U23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="V23" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="W23" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="R23" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S23" s="4" t="s">
+      <c r="X23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y23" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="T23" s="1" t="s">
+      <c r="Z23" s="1" t="s">
         <v>276</v>
-      </c>
-      <c r="U23" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V23" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="W23" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="X23" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y23" s="4" t="s">
-        <v>278</v>
-      </c>
-      <c r="Z23" s="1" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>28</v>
@@ -3504,13 +3498,13 @@
         <v>29</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>33</v>
@@ -3519,10 +3513,10 @@
         <v>34</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="L24" s="3" t="s">
         <v>37</v>
@@ -3541,7 +3535,7 @@
         <v>50</v>
       </c>
       <c r="T24" s="1" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="U24" s="3" t="s">
         <v>37</v>
@@ -3555,15 +3549,15 @@
         <v>50</v>
       </c>
       <c r="Z24" s="1" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="25" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>28</v>
@@ -3572,13 +3566,13 @@
         <v>29</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="H25" s="2" t="s">
         <v>33</v>
@@ -3587,10 +3581,10 @@
         <v>34</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>33</v>
@@ -3599,7 +3593,7 @@
         <v>29</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="O25" s="3" t="s">
         <v>37</v>
@@ -3615,10 +3609,10 @@
         <v>33</v>
       </c>
       <c r="V25" s="4" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="W25" s="1" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="X25" s="3" t="s">
         <v>37</v>
@@ -3628,25 +3622,25 @@
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D26" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="G26" s="1" t="s">
         <v>301</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>304</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>33</v>
@@ -3655,10 +3649,10 @@
         <v>34</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>37</v>
@@ -3679,10 +3673,10 @@
         <v>33</v>
       </c>
       <c r="V26" s="4" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="W26" s="1" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="X26" s="3" t="s">
         <v>37</v>
@@ -3692,10 +3686,10 @@
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>28</v>
@@ -3704,13 +3698,13 @@
         <v>29</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="H27" s="2" t="s">
         <v>33</v>
@@ -3719,10 +3713,10 @@
         <v>34</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>37</v>
@@ -3743,42 +3737,42 @@
         <v>33</v>
       </c>
       <c r="V27" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="W27" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="X27" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y27" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="Z27" s="1" t="s">
         <v>315</v>
-      </c>
-      <c r="W27" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="X27" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y27" s="4" t="s">
-        <v>317</v>
-      </c>
-      <c r="Z27" s="1" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="F28" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>33</v>
@@ -3787,10 +3781,10 @@
         <v>34</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="L28" s="3" t="s">
         <v>37</v>
@@ -3816,33 +3810,33 @@
         <v>33</v>
       </c>
       <c r="Y28" s="4" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="Z28" s="1" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="H29" s="2" t="s">
         <v>33</v>
@@ -3851,10 +3845,10 @@
         <v>34</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="L29" s="3" t="s">
         <v>37</v>
@@ -3880,33 +3874,33 @@
         <v>33</v>
       </c>
       <c r="Y29" s="4" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="Z29" s="1" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D30" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="G30" s="1" t="s">
         <v>356</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>357</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>359</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>33</v>
@@ -3915,10 +3909,10 @@
         <v>34</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="L30" s="3" t="s">
         <v>37</v>
@@ -3944,33 +3938,33 @@
         <v>33</v>
       </c>
       <c r="Y30" s="4" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="Z30" s="1" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
     </row>
     <row r="31" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>33</v>
@@ -3979,10 +3973,10 @@
         <v>34</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>37</v>
@@ -4011,30 +4005,30 @@
         <v>38</v>
       </c>
       <c r="Z31" s="1" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>33</v>
@@ -4043,10 +4037,10 @@
         <v>34</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="L32" s="3" t="s">
         <v>37</v>
@@ -4075,30 +4069,30 @@
         <v>38</v>
       </c>
       <c r="Z32" s="1" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="33" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="F33" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>33</v>
@@ -4107,10 +4101,10 @@
         <v>34</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="L33" s="3" t="s">
         <v>37</v>
@@ -4139,7 +4133,7 @@
         <v>38</v>
       </c>
       <c r="Z33" s="1" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
   </sheetData>
@@ -4171,13 +4165,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -4188,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>32</v>
@@ -4205,7 +4199,7 @@
         <v>41</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>46</v>
@@ -4222,7 +4216,7 @@
         <v>54</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>57</v>
@@ -4239,7 +4233,7 @@
         <v>65</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>69</v>
@@ -4256,7 +4250,7 @@
         <v>73</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>76</v>
@@ -4273,7 +4267,7 @@
         <v>85</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>88</v>
@@ -4290,7 +4284,7 @@
         <v>94</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>97</v>
@@ -4307,7 +4301,7 @@
         <v>104</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>107</v>
@@ -4324,10 +4318,10 @@
         <v>113</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>33</v>
@@ -4335,16 +4329,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>126</v>
-      </c>
       <c r="C11" s="4" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>33</v>
@@ -4352,16 +4346,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>134</v>
-      </c>
       <c r="C12" s="4" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>33</v>
@@ -4369,16 +4363,16 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>143</v>
-      </c>
       <c r="C13" s="4" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>33</v>
@@ -4386,16 +4380,16 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>154</v>
-      </c>
       <c r="C14" s="4" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>33</v>
@@ -4403,16 +4397,16 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>163</v>
-      </c>
       <c r="C15" s="4" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>33</v>
@@ -4420,16 +4414,16 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>176</v>
-      </c>
       <c r="C16" s="4" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>33</v>
@@ -4437,16 +4431,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>187</v>
-      </c>
       <c r="C17" s="4" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>33</v>
@@ -4454,16 +4448,16 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>199</v>
-      </c>
       <c r="C18" s="4" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>33</v>
@@ -4471,16 +4465,16 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>210</v>
-      </c>
       <c r="C19" s="4" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>33</v>
@@ -4488,16 +4482,16 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>33</v>
@@ -4505,16 +4499,16 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>33</v>
@@ -4522,16 +4516,16 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>246</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>248</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>33</v>
@@ -4539,16 +4533,16 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>33</v>
@@ -4556,16 +4550,16 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>33</v>
@@ -4573,16 +4567,16 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B25" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>281</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>421</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>284</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>33</v>
@@ -4590,16 +4584,16 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B26" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>290</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>293</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>33</v>
@@ -4607,16 +4601,16 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>33</v>
@@ -4624,16 +4618,16 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="B28" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>309</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>312</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>33</v>
@@ -4641,16 +4635,16 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="E29" s="7" t="s">
         <v>33</v>
@@ -4658,16 +4652,16 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B30" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>423</v>
+      </c>
+      <c r="D30" s="4" t="s">
         <v>330</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>426</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>333</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>33</v>
@@ -4675,16 +4669,16 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B31" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D31" s="4" t="s">
         <v>339</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>427</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>342</v>
       </c>
       <c r="E31" s="7" t="s">
         <v>33</v>
@@ -4692,16 +4686,16 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B32" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="D32" s="4" t="s">
         <v>347</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>428</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>350</v>
       </c>
       <c r="E32" s="7" t="s">
         <v>33</v>
@@ -4709,16 +4703,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="E33" s="7" t="s">
         <v>33</v>
@@ -4726,16 +4720,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B34" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="D34" s="4" t="s">
         <v>364</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>430</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>367</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>33</v>
@@ -4743,16 +4737,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="D35" s="4" t="s">
         <v>371</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>372</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>431</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>374</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>33</v>
@@ -4760,16 +4754,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="D36" s="4" t="s">
         <v>378</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>432</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>433</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>381</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>33</v>
@@ -4777,16 +4771,16 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B37" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="D37" s="4" t="s">
         <v>386</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>434</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>389</v>
       </c>
       <c r="E37" s="7" t="s">
         <v>33</v>
@@ -4992,25 +4986,25 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>101</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>321</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>323</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>324</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>33</v>
@@ -5019,10 +5013,10 @@
         <v>34</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>37</v>
@@ -5038,10 +5032,10 @@
         <v>33</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="U3" s="3" t="s">
         <v>37</v>
@@ -5052,33 +5046,33 @@
         <v>33</v>
       </c>
       <c r="Y3" s="4" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>101</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>33</v>
@@ -5087,10 +5081,10 @@
         <v>34</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>37</v>
@@ -5106,10 +5100,10 @@
         <v>33</v>
       </c>
       <c r="S4" s="4" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="U4" s="3" t="s">
         <v>37</v>
@@ -5120,33 +5114,33 @@
         <v>33</v>
       </c>
       <c r="Y4" s="4" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>101</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>33</v>
@@ -5155,10 +5149,10 @@
         <v>34</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>37</v>
@@ -5174,10 +5168,10 @@
         <v>33</v>
       </c>
       <c r="S5" s="4" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="U5" s="3" t="s">
         <v>37</v>
@@ -5188,10 +5182,10 @@
         <v>33</v>
       </c>
       <c r="Y5" s="4" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly sync 2026-06-09: Osama Al-Zamil bio title, two Legal Counsel fixes, Osama Al-Thanon email (#34)
Co-authored-by: Taranis Sync Bot <sync@taraniscapital.com>
</commit_message>
<xml_diff>
--- a/Taranis-People-Data-Collection.xlsx
+++ b/Taranis-People-Data-Collection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mark\Claude Cowork\Taranis Capital Website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C187EC5-08D0-428A-9135-9CD47602A1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7AEFF62-1B67-497A-B4C9-6606C5236166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="People Directory" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="435">
   <si>
     <t>Slug</t>
   </si>
@@ -384,9 +384,6 @@
     <t>Emad Zowawi</t>
   </si>
   <si>
-    <t>KSA Legal Consul to the CEO</t>
-  </si>
-  <si>
     <t>emad@taraniscapital.com</t>
   </si>
   <si>
@@ -681,9 +678,6 @@
     <t>Mohamed Essam</t>
   </si>
   <si>
-    <t>Legal Consul</t>
-  </si>
-  <si>
     <t>mohamed@taraniscapital.com</t>
   </si>
   <si>
@@ -829,10 +823,6 @@
     <t>/images/team/His-Excellency-Eng.-Osama-Abdulaziz-Al-Zamil-Joins-600x650-1-277x300.png</t>
   </si>
   <si>
-    <t>Osama Al-Zamil is Chairman of the Advisory Board at Taranis Capital. He is a distinguished Saudi industrial leader with a remarkable career spanning multiple decades in business, government, and strategic advisory roles.
-His extensive experience includes senior government positions, including former Vice Minister of Industry, as well as leadership roles in major Saudi industrial and commercial enterprises. He brings unparalleled expertise in MENA markets, industrial development, international trade, and strategic capital deployment.</t>
-  </si>
-  <si>
     <t>taraniscapital.com/board/osama-al-zamil</t>
   </si>
   <si>
@@ -1389,6 +1379,10 @@
   </si>
   <si>
     <t>Chief Strategy Officer</t>
+  </si>
+  <si>
+    <t>Osama Al-Zamil is a Board Adviser at Taranis Capital. He is a distinguished Saudi industrial leader with a remarkable career spanning multiple decades in business, government, and strategic advisory roles.
+His extensive experience includes senior government positions, including former Vice Minister of Industry, as well as leadership roles in major Saudi industrial and commercial enterprises. He brings unparalleled expertise in MENA markets, industrial development, international trade, and strategic capital deployment.</t>
   </si>
 </sst>
 </file>
@@ -2405,16 +2399,16 @@
         <v>42</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>33</v>
@@ -2423,10 +2417,10 @@
         <v>34</v>
       </c>
       <c r="J9" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="K9" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>37</v>
@@ -2437,19 +2431,19 @@
         <v>33</v>
       </c>
       <c r="P9" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q9" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="Q9" s="1" t="s">
+      <c r="R9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S9" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="R9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S9" s="4" t="s">
+      <c r="T9" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>123</v>
       </c>
       <c r="U9" s="3" t="s">
         <v>37</v>
@@ -2460,18 +2454,18 @@
         <v>33</v>
       </c>
       <c r="Y9" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="Z9" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>126</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>28</v>
@@ -2480,13 +2474,13 @@
         <v>29</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>33</v>
@@ -2495,10 +2489,10 @@
         <v>34</v>
       </c>
       <c r="J10" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="K10" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>130</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>37</v>
@@ -2514,10 +2508,10 @@
         <v>33</v>
       </c>
       <c r="S10" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="T10" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="T10" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="U10" s="3" t="s">
         <v>37</v>
@@ -2532,10 +2526,10 @@
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>134</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>28</v>
@@ -2544,13 +2538,13 @@
         <v>29</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>137</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>33</v>
@@ -2559,10 +2553,10 @@
         <v>34</v>
       </c>
       <c r="J11" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="K11" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>139</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>33</v>
@@ -2571,7 +2565,7 @@
         <v>29</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O11" s="3" t="s">
         <v>37</v>
@@ -2590,7 +2584,7 @@
         <v>29</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="X11" s="3" t="s">
         <v>37</v>
@@ -2600,10 +2594,10 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>143</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>28</v>
@@ -2612,13 +2606,13 @@
         <v>29</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>33</v>
@@ -2627,10 +2621,10 @@
         <v>34</v>
       </c>
       <c r="J12" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="K12" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>148</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>33</v>
@@ -2639,16 +2633,16 @@
         <v>29</v>
       </c>
       <c r="N12" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P12" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="O12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P12" s="4" t="s">
+      <c r="Q12" s="1" t="s">
         <v>150</v>
-      </c>
-      <c r="Q12" s="1" t="s">
-        <v>151</v>
       </c>
       <c r="R12" s="3" t="s">
         <v>37</v>
@@ -2662,7 +2656,7 @@
         <v>29</v>
       </c>
       <c r="W12" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="X12" s="3" t="s">
         <v>37</v>
@@ -2672,10 +2666,10 @@
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>28</v>
@@ -2684,13 +2678,13 @@
         <v>29</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>156</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>157</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>33</v>
@@ -2699,10 +2693,10 @@
         <v>34</v>
       </c>
       <c r="J13" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="K13" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="L13" s="3" t="s">
         <v>37</v>
@@ -2718,10 +2712,10 @@
         <v>33</v>
       </c>
       <c r="S13" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="T13" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="T13" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="U13" s="3" t="s">
         <v>37</v>
@@ -2736,25 +2730,25 @@
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>163</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>167</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>33</v>
@@ -2763,63 +2757,63 @@
         <v>34</v>
       </c>
       <c r="J14" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="K14" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="L14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M14" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="N14" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="L14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M14" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="N14" s="1" t="s">
+      <c r="O14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="Q14" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="O14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P14" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="Q14" s="1" t="s">
+      <c r="R14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S14" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="T14" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="R14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S14" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="T14" s="1" t="s">
+      <c r="U14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="V14" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="W14" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="U14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V14" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="W14" s="1" t="s">
+      <c r="X14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y14" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="Z14" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="X14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y14" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="Z14" s="1" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>176</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>28</v>
@@ -2828,13 +2822,13 @@
         <v>29</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>179</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>33</v>
@@ -2843,10 +2837,10 @@
         <v>34</v>
       </c>
       <c r="J15" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="K15" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>181</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>37</v>
@@ -2857,19 +2851,19 @@
         <v>33</v>
       </c>
       <c r="P15" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="Q15" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="R15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S15" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="T15" s="1" t="s">
         <v>182</v>
-      </c>
-      <c r="R15" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S15" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="T15" s="1" t="s">
-        <v>183</v>
       </c>
       <c r="U15" s="3" t="s">
         <v>37</v>
@@ -2880,18 +2874,18 @@
         <v>33</v>
       </c>
       <c r="Y15" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="Z15" s="1" t="s">
         <v>184</v>
-      </c>
-      <c r="Z15" s="1" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>186</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>187</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>28</v>
@@ -2900,13 +2894,13 @@
         <v>29</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>33</v>
@@ -2915,10 +2909,10 @@
         <v>34</v>
       </c>
       <c r="J16" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="K16" s="1" t="s">
         <v>191</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>33</v>
@@ -2927,7 +2921,7 @@
         <v>29</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O16" s="3" t="s">
         <v>33</v>
@@ -2936,7 +2930,7 @@
         <v>50</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="R16" s="3" t="s">
         <v>33</v>
@@ -2945,7 +2939,7 @@
         <v>50</v>
       </c>
       <c r="T16" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="U16" s="3" t="s">
         <v>33</v>
@@ -2954,7 +2948,7 @@
         <v>29</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="X16" s="3" t="s">
         <v>33</v>
@@ -2963,30 +2957,30 @@
         <v>50</v>
       </c>
       <c r="Z16" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>198</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>199</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>33</v>
@@ -2995,10 +2989,10 @@
         <v>34</v>
       </c>
       <c r="J17" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="K17" s="1" t="s">
         <v>204</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>205</v>
       </c>
       <c r="L17" s="3" t="s">
         <v>37</v>
@@ -3014,19 +3008,19 @@
         <v>33</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="T17" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="U17" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="V17" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="U17" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V17" s="4" t="s">
+      <c r="W17" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="W17" s="1" t="s">
-        <v>208</v>
       </c>
       <c r="X17" s="3" t="s">
         <v>37</v>
@@ -3036,25 +3030,25 @@
     </row>
     <row r="18" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>210</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>214</v>
       </c>
       <c r="H18" s="2" t="s">
         <v>33</v>
@@ -3063,78 +3057,78 @@
         <v>34</v>
       </c>
       <c r="J18" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M18" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="N18" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="L18" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M18" s="4" t="s">
+      <c r="O18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P18" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q18" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="N18" s="1" t="s">
+      <c r="R18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S18" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="T18" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="O18" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P18" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="Q18" s="1" t="s">
+      <c r="U18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="V18" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="W18" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="R18" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S18" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="T18" s="1" t="s">
+      <c r="X18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y18" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="Z18" s="1" t="s">
         <v>220</v>
-      </c>
-      <c r="U18" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V18" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="W18" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="X18" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y18" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="Z18" s="1" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="19" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>33</v>
@@ -3143,10 +3137,10 @@
         <v>34</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>37</v>
@@ -3172,33 +3166,33 @@
         <v>33</v>
       </c>
       <c r="Y19" s="4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="Z19" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="20" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>235</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>237</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>33</v>
@@ -3207,78 +3201,78 @@
         <v>34</v>
       </c>
       <c r="J20" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="N20" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="K20" s="1" t="s">
+      <c r="O20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P20" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="Q20" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="L20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M20" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="N20" s="1" t="s">
+      <c r="R20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S20" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="T20" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="O20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P20" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="Q20" s="1" t="s">
+      <c r="U20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="V20" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="W20" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="X20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y20" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="R20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S20" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="T20" s="1" t="s">
+      <c r="Z20" s="1" t="s">
         <v>242</v>
-      </c>
-      <c r="U20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V20" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="W20" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="X20" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y20" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="Z20" s="1" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="21" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>33</v>
@@ -3287,19 +3281,19 @@
         <v>34</v>
       </c>
       <c r="J21" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M21" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="N21" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="L21" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M21" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="N21" s="1" t="s">
-        <v>251</v>
       </c>
       <c r="O21" s="3" t="s">
         <v>37</v>
@@ -3310,10 +3304,10 @@
         <v>33</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="T21" s="1" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="U21" s="3" t="s">
         <v>33</v>
@@ -3322,7 +3316,7 @@
         <v>29</v>
       </c>
       <c r="W21" s="1" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="X21" s="3" t="s">
         <v>33</v>
@@ -3331,30 +3325,30 @@
         <v>50</v>
       </c>
       <c r="Z21" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>33</v>
@@ -3363,10 +3357,10 @@
         <v>34</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>259</v>
+        <v>434</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="L22" s="3" t="s">
         <v>37</v>
@@ -3380,7 +3374,7 @@
         <v>50</v>
       </c>
       <c r="Q22" s="1" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="R22" s="3" t="s">
         <v>33</v>
@@ -3389,7 +3383,7 @@
         <v>50</v>
       </c>
       <c r="T22" s="1" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="U22" s="3" t="s">
         <v>33</v>
@@ -3398,7 +3392,7 @@
         <v>50</v>
       </c>
       <c r="W22" s="1" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="X22" s="3" t="s">
         <v>33</v>
@@ -3407,30 +3401,30 @@
         <v>50</v>
       </c>
       <c r="Z22" s="1" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="23" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D23" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="G23" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>270</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>33</v>
@@ -3439,63 +3433,63 @@
         <v>34</v>
       </c>
       <c r="J23" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M23" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="O23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P23" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="Q23" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="K23" s="1" t="s">
+      <c r="R23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="S23" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="L23" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M23" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="N23" s="1" t="s">
+      <c r="T23" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="O23" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P23" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="Q23" s="1" t="s">
+      <c r="U23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="V23" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="W23" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="R23" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="S23" s="4" t="s">
+      <c r="X23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y23" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="T23" s="1" t="s">
+      <c r="Z23" s="1" t="s">
         <v>276</v>
-      </c>
-      <c r="U23" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="V23" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="W23" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="X23" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y23" s="4" t="s">
-        <v>278</v>
-      </c>
-      <c r="Z23" s="1" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>28</v>
@@ -3504,13 +3498,13 @@
         <v>29</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>33</v>
@@ -3519,10 +3513,10 @@
         <v>34</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="L24" s="3" t="s">
         <v>37</v>
@@ -3541,7 +3535,7 @@
         <v>50</v>
       </c>
       <c r="T24" s="1" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="U24" s="3" t="s">
         <v>37</v>
@@ -3555,15 +3549,15 @@
         <v>50</v>
       </c>
       <c r="Z24" s="1" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="25" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>28</v>
@@ -3572,13 +3566,13 @@
         <v>29</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="H25" s="2" t="s">
         <v>33</v>
@@ -3587,10 +3581,10 @@
         <v>34</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>33</v>
@@ -3599,7 +3593,7 @@
         <v>29</v>
       </c>
       <c r="N25" s="1" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="O25" s="3" t="s">
         <v>37</v>
@@ -3615,10 +3609,10 @@
         <v>33</v>
       </c>
       <c r="V25" s="4" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="W25" s="1" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="X25" s="3" t="s">
         <v>37</v>
@@ -3628,25 +3622,25 @@
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>42</v>
       </c>
       <c r="D26" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="G26" s="1" t="s">
         <v>301</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>304</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>33</v>
@@ -3655,10 +3649,10 @@
         <v>34</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>37</v>
@@ -3679,10 +3673,10 @@
         <v>33</v>
       </c>
       <c r="V26" s="4" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="W26" s="1" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="X26" s="3" t="s">
         <v>37</v>
@@ -3692,10 +3686,10 @@
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>28</v>
@@ -3704,13 +3698,13 @@
         <v>29</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="H27" s="2" t="s">
         <v>33</v>
@@ -3719,10 +3713,10 @@
         <v>34</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>37</v>
@@ -3743,42 +3737,42 @@
         <v>33</v>
       </c>
       <c r="V27" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="W27" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="X27" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y27" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="Z27" s="1" t="s">
         <v>315</v>
-      </c>
-      <c r="W27" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="X27" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y27" s="4" t="s">
-        <v>317</v>
-      </c>
-      <c r="Z27" s="1" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="F28" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>33</v>
@@ -3787,10 +3781,10 @@
         <v>34</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="L28" s="3" t="s">
         <v>37</v>
@@ -3816,33 +3810,33 @@
         <v>33</v>
       </c>
       <c r="Y28" s="4" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="Z28" s="1" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="H29" s="2" t="s">
         <v>33</v>
@@ -3851,10 +3845,10 @@
         <v>34</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="L29" s="3" t="s">
         <v>37</v>
@@ -3880,33 +3874,33 @@
         <v>33</v>
       </c>
       <c r="Y29" s="4" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="Z29" s="1" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D30" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="G30" s="1" t="s">
         <v>356</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>357</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>359</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>33</v>
@@ -3915,10 +3909,10 @@
         <v>34</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="L30" s="3" t="s">
         <v>37</v>
@@ -3944,33 +3938,33 @@
         <v>33</v>
       </c>
       <c r="Y30" s="4" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="Z30" s="1" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
     </row>
     <row r="31" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>33</v>
@@ -3979,10 +3973,10 @@
         <v>34</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>37</v>
@@ -4011,30 +4005,30 @@
         <v>38</v>
       </c>
       <c r="Z31" s="1" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>33</v>
@@ -4043,10 +4037,10 @@
         <v>34</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="L32" s="3" t="s">
         <v>37</v>
@@ -4075,30 +4069,30 @@
         <v>38</v>
       </c>
       <c r="Z32" s="1" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="33" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="F33" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>33</v>
@@ -4107,10 +4101,10 @@
         <v>34</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="L33" s="3" t="s">
         <v>37</v>
@@ -4139,7 +4133,7 @@
         <v>38</v>
       </c>
       <c r="Z33" s="1" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
   </sheetData>
@@ -4171,13 +4165,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -4188,7 +4182,7 @@
         <v>27</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>32</v>
@@ -4205,7 +4199,7 @@
         <v>41</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>46</v>
@@ -4222,7 +4216,7 @@
         <v>54</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>57</v>
@@ -4239,7 +4233,7 @@
         <v>65</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>69</v>
@@ -4256,7 +4250,7 @@
         <v>73</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>76</v>
@@ -4273,7 +4267,7 @@
         <v>85</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>88</v>
@@ -4290,7 +4284,7 @@
         <v>94</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>97</v>
@@ -4307,7 +4301,7 @@
         <v>104</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>107</v>
@@ -4324,10 +4318,10 @@
         <v>113</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>33</v>
@@ -4335,16 +4329,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>126</v>
-      </c>
       <c r="C11" s="4" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>33</v>
@@ -4352,16 +4346,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>134</v>
-      </c>
       <c r="C12" s="4" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>33</v>
@@ -4369,16 +4363,16 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>143</v>
-      </c>
       <c r="C13" s="4" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>33</v>
@@ -4386,16 +4380,16 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>154</v>
-      </c>
       <c r="C14" s="4" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>33</v>
@@ -4403,16 +4397,16 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>163</v>
-      </c>
       <c r="C15" s="4" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>33</v>
@@ -4420,16 +4414,16 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>176</v>
-      </c>
       <c r="C16" s="4" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>33</v>
@@ -4437,16 +4431,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>187</v>
-      </c>
       <c r="C17" s="4" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>33</v>
@@ -4454,16 +4448,16 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>199</v>
-      </c>
       <c r="C18" s="4" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>33</v>
@@ -4471,16 +4465,16 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>210</v>
-      </c>
       <c r="C19" s="4" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>33</v>
@@ -4488,16 +4482,16 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>33</v>
@@ -4505,16 +4499,16 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>33</v>
@@ -4522,16 +4516,16 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>246</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>248</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>33</v>
@@ -4539,16 +4533,16 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>33</v>
@@ -4556,16 +4550,16 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>33</v>
@@ -4573,16 +4567,16 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B25" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>281</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>421</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>284</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>33</v>
@@ -4590,16 +4584,16 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B26" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>290</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>422</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>293</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>33</v>
@@ -4607,16 +4601,16 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>33</v>
@@ -4624,16 +4618,16 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="B28" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>309</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>424</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>312</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>33</v>
@@ -4641,16 +4635,16 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="E29" s="7" t="s">
         <v>33</v>
@@ -4658,16 +4652,16 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B30" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>423</v>
+      </c>
+      <c r="D30" s="4" t="s">
         <v>330</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>426</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>333</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>33</v>
@@ -4675,16 +4669,16 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B31" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="D31" s="4" t="s">
         <v>339</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>427</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>342</v>
       </c>
       <c r="E31" s="7" t="s">
         <v>33</v>
@@ -4692,16 +4686,16 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B32" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="D32" s="4" t="s">
         <v>347</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>428</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>350</v>
       </c>
       <c r="E32" s="7" t="s">
         <v>33</v>
@@ -4709,16 +4703,16 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="E33" s="7" t="s">
         <v>33</v>
@@ -4726,16 +4720,16 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B34" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="D34" s="4" t="s">
         <v>364</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>430</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>367</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>33</v>
@@ -4743,16 +4737,16 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="D35" s="4" t="s">
         <v>371</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>372</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>431</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>374</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>33</v>
@@ -4760,16 +4754,16 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="D36" s="4" t="s">
         <v>378</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>432</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>433</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>381</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>33</v>
@@ -4777,16 +4771,16 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B37" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="D37" s="4" t="s">
         <v>386</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>434</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>389</v>
       </c>
       <c r="E37" s="7" t="s">
         <v>33</v>
@@ -4992,25 +4986,25 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>101</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>321</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>323</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>324</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>33</v>
@@ -5019,10 +5013,10 @@
         <v>34</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>37</v>
@@ -5038,10 +5032,10 @@
         <v>33</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="U3" s="3" t="s">
         <v>37</v>
@@ -5052,33 +5046,33 @@
         <v>33</v>
       </c>
       <c r="Y3" s="4" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>101</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>33</v>
@@ -5087,10 +5081,10 @@
         <v>34</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>37</v>
@@ -5106,10 +5100,10 @@
         <v>33</v>
       </c>
       <c r="S4" s="4" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="U4" s="3" t="s">
         <v>37</v>
@@ -5120,33 +5114,33 @@
         <v>33</v>
       </c>
       <c r="Y4" s="4" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>101</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>87</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>33</v>
@@ -5155,10 +5149,10 @@
         <v>34</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>37</v>
@@ -5174,10 +5168,10 @@
         <v>33</v>
       </c>
       <c r="S5" s="4" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="U5" s="3" t="s">
         <v>37</v>
@@ -5188,10 +5182,10 @@
         <v>33</v>
       </c>
       <c r="Y5" s="4" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
   </sheetData>

</xml_diff>